<commit_message>
update template firm order
</commit_message>
<xml_diff>
--- a/RFIDP2P3_Web/wwwroot/templates/Firm Tentative Order.xlsx
+++ b/RFIDP2P3_Web/wwwroot/templates/Firm Tentative Order.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\webproject\RFID-Anbunka-Frontend\RFIDP2P3_Web\wwwroot\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6531B5B1-705B-4FDB-A996-96DF6A515771}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A244BFF-93B4-4085-8DEA-A204975F0D59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="12196" xr2:uid="{50EC5814-6AD7-4EEB-B009-21B13A67DEED}"/>
   </bookViews>
@@ -24,40 +24,6 @@
 </workbook>
 </file>
 
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author>Henry Hartawan</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{2EB2CEEA-F84D-4128-B6B4-7B5ED6E6F6CE}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>ICS:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-harus dalam format cells = text</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
@@ -95,7 +61,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -123,19 +89,6 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -480,7 +433,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{645F3AD8-7DA3-489A-AD94-02784AC6392B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{645F3AD8-7DA3-489A-AD94-02784AC6392B}">
   <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
@@ -537,6 +490,5 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>